<commit_message>
Commiting & pushing for backup purposes
</commit_message>
<xml_diff>
--- a/Salaray_Breakdown_Analysis.xlsx
+++ b/Salaray_Breakdown_Analysis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git_Repositories\PubDev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC7F87A5-37AC-4D55-BFE7-6AA4CE676CA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EE71685-D80C-4DE7-93B8-E481C896C4C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="39810" yWindow="2415" windowWidth="35595" windowHeight="15345" xr2:uid="{5DEC0479-A997-4C84-988A-5D2FAA7FE317}"/>
+    <workbookView xWindow="2340" yWindow="1830" windowWidth="30285" windowHeight="15345" xr2:uid="{5DEC0479-A997-4C84-988A-5D2FAA7FE317}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>Fuel economy (mile / gal)</t>
   </si>
@@ -87,18 +87,6 @@
     <t>Weekly car wash ($)</t>
   </si>
   <si>
-    <t>Fuel</t>
-  </si>
-  <si>
-    <t>Oil</t>
-  </si>
-  <si>
-    <t>Brakes</t>
-  </si>
-  <si>
-    <t>Misc Auto</t>
-  </si>
-  <si>
     <t>Gross annual pay ($)</t>
   </si>
   <si>
@@ -120,20 +108,23 @@
     <t>Pay Related</t>
   </si>
   <si>
-    <t>Health Insurance Related</t>
-  </si>
-  <si>
     <t>Weekly Out-Of-Pocket</t>
   </si>
   <si>
     <t>Emotional Wear Coefficient</t>
+  </si>
+  <si>
+    <t>Vehicle Related</t>
+  </si>
+  <si>
+    <t>Weekly pay ($)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -148,12 +139,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -233,11 +218,11 @@
     <xf numFmtId="40" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+      <alignment horizontal="right" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -587,7 +572,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD21BCDC-0F36-4605-9774-C1621DC87D5B}">
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" bestFit="1" customWidth="1"/>
@@ -600,15 +585,15 @@
   <sheetData>
     <row r="1" spans="1:10" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="B1" s="2"/>
       <c r="E1" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F1" s="2"/>
       <c r="I1" s="1" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="J1" s="2"/>
     </row>
@@ -620,14 +605,14 @@
         <v>4.5</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F2" s="4">
         <f>45*2</f>
         <v>90</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="J2" s="4">
         <v>130000</v>
@@ -641,13 +626,13 @@
         <v>42</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F3" s="6">
         <v>5</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="J3" s="6">
         <f>J2/2080</f>
@@ -655,98 +640,82 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="E4" s="8" t="s">
-        <v>18</v>
+      <c r="A4" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4">
+        <v>3000</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>14</v>
       </c>
       <c r="F4" s="4">
         <f>F2*F3*52</f>
         <v>23400</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="2"/>
+      <c r="I4" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="J4" s="4"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="6">
+        <f>(((4.2/12)*60)*4.2)+15</f>
+        <v>103.20000000000002</v>
+      </c>
       <c r="E5" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="F5" s="6">
         <v>0</v>
       </c>
-      <c r="I5" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="J5" s="2"/>
+      <c r="I5" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="J5" s="6">
+        <v>1200</v>
+      </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>2</v>
+      <c r="A6" s="7" t="s">
+        <v>4</v>
       </c>
       <c r="B6" s="4">
-        <v>3000</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J6" s="4"/>
+        <v>650</v>
+      </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B7" s="6">
-        <f>(((4.2/12)*60)*4.2)+15</f>
-        <v>103.20000000000002</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B9" s="2"/>
+        <v>75000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="6">
+        <v>60000</v>
+      </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B10" s="4"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B11" s="6"/>
-    </row>
-    <row r="13" spans="1:10" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" s="2"/>
-    </row>
-    <row r="14" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B14" s="4"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B15" s="6"/>
-    </row>
-    <row r="17" spans="1:2" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B17" s="2"/>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
+      <c r="A10" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B18" s="4">
+      <c r="B10" s="4">
         <f>40/4</f>
         <v>10</v>
       </c>

</xml_diff>